<commit_message>
Auto healing Report implementation done
</commit_message>
<xml_diff>
--- a/EaTestAutomation/TestData/TestData.xlsx
+++ b/EaTestAutomation/TestData/TestData.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DEMO Project\EaTestAutomation\TestData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EaAutomationFramework\EaTestAutomation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66BD3C00-BA78-4563-BC57-780FF6D77C78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C26CCDE0-B18B-423C-9D3A-26C0AA59A76A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -485,7 +485,7 @@
         <v>8</v>
       </c>
       <c r="B2" s="1">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C2" s="1">
         <v>10000</v>
@@ -602,7 +602,7 @@
         <v>12</v>
       </c>
       <c r="B2" s="1">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C2" s="1">
         <v>10000</v>

</xml_diff>

<commit_message>
Parallel run implementation done and Dashboard artifact issue resolved
</commit_message>
<xml_diff>
--- a/EaTestAutomation/TestData/TestData.xlsx
+++ b/EaTestAutomation/TestData/TestData.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EaAutomationFramework\EaTestAutomation\TestData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\EaAutomationFramework\EaTestAutomation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49C07711-F46F-41FB-9105-9223E4C64BC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E6B84A1-1B82-4BF3-93E7-5B5E6032EE96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AddNewEmployee" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="15">
   <si>
     <t>Name</t>
   </si>
@@ -60,6 +60,12 @@
   </si>
   <si>
     <t>Raj</t>
+  </si>
+  <si>
+    <t>PASS</t>
+  </si>
+  <si>
+    <t/>
   </si>
 </sst>
 </file>
@@ -413,20 +419,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:J3"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.7265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="3.90625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.90625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.6328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.7265625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.36328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.36328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="3.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -451,8 +457,14 @@
       <c r="H1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I1" t="s">
+        <v>6</v>
+      </c>
+      <c r="J1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
@@ -474,8 +486,14 @@
       <c r="G2" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -494,14 +512,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="16" width="9.1796875" customWidth="1"/>
-    <col min="17" max="20" width="9.08984375" customWidth="1"/>
+    <col min="1" max="5" width="9.21875" customWidth="1"/>
+    <col min="6" max="6" width="15.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="16" width="9.21875" customWidth="1"/>
+    <col min="17" max="20" width="9.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -521,7 +541,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>12</v>
       </c>
@@ -529,10 +549,10 @@
         <v>27</v>
       </c>
       <c r="C2" s="1">
-        <v>11000</v>
+        <v>110001</v>
       </c>
       <c r="D2" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>9</v>
@@ -541,17 +561,72 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="1">
+        <v>28</v>
+      </c>
+      <c r="C3" s="1">
+        <v>110002</v>
+      </c>
+      <c r="D3" s="1">
+        <v>2</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="1">
+        <v>29</v>
+      </c>
+      <c r="C4" s="1">
+        <v>110003</v>
+      </c>
+      <c r="D4" s="1">
+        <v>4</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="1">
+        <v>30</v>
+      </c>
+      <c r="C5" s="1">
+        <v>110004</v>
+      </c>
+      <c r="D5" s="1">
+        <v>3</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>10</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="F2" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
+    <hyperlink ref="F3" r:id="rId2" xr:uid="{396EF4D6-934D-447F-8348-57E636E6AC20}"/>
+    <hyperlink ref="F4" r:id="rId3" xr:uid="{F9E1D243-F3DB-4439-BFCA-067534308E1F}"/>
+    <hyperlink ref="F5" r:id="rId4" xr:uid="{F69B0E32-C330-44B5-BB7D-409839230CC0}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Framework Locators healing issue Fix
</commit_message>
<xml_diff>
--- a/EaTestAutomation/TestData/TestData.xlsx
+++ b/EaTestAutomation/TestData/TestData.xlsx
@@ -45,6 +45,12 @@
     <x:t>TestResult</x:t>
   </x:si>
   <x:si>
+    <x:t>Reference</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Message</x:t>
+  </x:si>
+  <x:si>
     <x:t>ErrorMessage</x:t>
   </x:si>
   <x:si>
@@ -57,25 +63,13 @@
     <x:t>Test2@gmail.com</x:t>
   </x:si>
   <x:si>
-    <x:t>FAIL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PASS</x:t>
+    <x:t>Pass</x:t>
   </x:si>
   <x:si>
     <x:t/>
   </x:si>
   <x:si>
     <x:t>Raj</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Reference</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Message</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Pass</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -461,6 +455,7 @@
     <x:col min="6" max="6" width="15.664062" style="0" bestFit="1" customWidth="1"/>
     <x:col min="7" max="7" width="9.332031" style="0" bestFit="1" customWidth="1"/>
     <x:col min="8" max="8" width="12.332031" style="0" bestFit="1" customWidth="1"/>
+    <x:col min="9" max="10" width="9.139196" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:10" x14ac:dyDescent="0.3">
@@ -489,15 +484,15 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="I1" s="0" t="s">
-        <x:v>6</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="J1" s="0" t="s">
-        <x:v>7</x:v>
+        <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <x:c r="A2" s="1" t="s">
-        <x:v>8</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B2" s="1">
         <x:v>23</x:v>
@@ -509,19 +504,22 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="E2" s="1" t="s">
-        <x:v>9</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="F2" s="3" t="s">
-        <x:v>10</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="G2" s="0" t="s">
-        <x:v>11</x:v>
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="H2" s="0" t="s">
+        <x:v>12</x:v>
       </x:c>
       <x:c r="I2" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="J2" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:10" x14ac:dyDescent="0.3">
@@ -534,7 +532,7 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink ref="F2" r:id="rId6"/>
+    <x:hyperlink ref="F2" r:id="rId16"/>
   </x:hyperlinks>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -581,15 +579,15 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="H1" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="I1" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:20" x14ac:dyDescent="0.3">
       <x:c r="A2" s="1" t="s">
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="B2" s="1">
         <x:v>27</x:v>
@@ -601,15 +599,24 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E2" s="1" t="s">
-        <x:v>9</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="F2" s="3" t="s">
-        <x:v>10</x:v>
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="G2" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="H2" s="0" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="I2" s="0" t="s">
+        <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:20" x14ac:dyDescent="0.3">
       <x:c r="A3" s="1" t="s">
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="B3" s="1">
         <x:v>28</x:v>
@@ -621,24 +628,24 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="E3" s="1" t="s">
-        <x:v>9</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="F3" s="3" t="s">
-        <x:v>10</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="G3" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="H3" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="I3" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:20" x14ac:dyDescent="0.3">
       <x:c r="A4" s="1" t="s">
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="B4" s="1">
         <x:v>29</x:v>
@@ -650,15 +657,24 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="E4" s="1" t="s">
-        <x:v>9</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="F4" s="3" t="s">
-        <x:v>10</x:v>
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="G4" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="H4" s="0" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="I4" s="0" t="s">
+        <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:20" x14ac:dyDescent="0.3">
       <x:c r="A5" s="1" t="s">
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="B5" s="1">
         <x:v>30</x:v>
@@ -670,18 +686,27 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="E5" s="1" t="s">
-        <x:v>9</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="F5" s="3" t="s">
-        <x:v>10</x:v>
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="G5" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="H5" s="0" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="I5" s="0" t="s">
+        <x:v>14</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink ref="F2" r:id="rId7"/>
-    <x:hyperlink ref="F3" r:id="rId8"/>
-    <x:hyperlink ref="F4" r:id="rId9"/>
-    <x:hyperlink ref="F5" r:id="rId10"/>
+    <x:hyperlink ref="F2" r:id="rId17"/>
+    <x:hyperlink ref="F3" r:id="rId18"/>
+    <x:hyperlink ref="F4" r:id="rId19"/>
+    <x:hyperlink ref="F5" r:id="rId20"/>
   </x:hyperlinks>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>